<commit_message>
更新网站内容 - 2026-05-01 16:32:50
</commit_message>
<xml_diff>
--- a/hexo/hexo/public/account-display/ta/作品列表.xlsx
+++ b/hexo/hexo/public/account-display/ta/作品列表.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="239">
   <si>
     <t>作品名称</t>
   </si>
@@ -66,40 +66,103 @@
     <t>粉丝增量</t>
   </si>
   <si>
+    <t>AI这么火，为什么一堆公司倒闭了？#科技下一站 #还有什么是不能ai的 #与ai同行 #大模型 #行业大揭秘</t>
+  </si>
+  <si>
+    <t>2026-04-30 22:40:21</t>
+  </si>
+  <si>
+    <t>1-3min视频</t>
+  </si>
+  <si>
+    <t>公开</t>
+  </si>
+  <si>
+    <t>402</t>
+  </si>
+  <si>
+    <t>0.035714</t>
+  </si>
+  <si>
+    <t>0.529716</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>0.284238</t>
+  </si>
+  <si>
+    <t>21.534146</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>AI不会取代你的工作，但会用AI的人会 #AI焦虑 #自动化办公 #科技改变生活 #大模型</t>
+  </si>
+  <si>
+    <t>2026-04-30 22:00:53</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>0.046154</t>
+  </si>
+  <si>
+    <t>0.202703</t>
+  </si>
+  <si>
+    <t>0.608108</t>
+  </si>
+  <si>
+    <t>9.729730</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>普通人上大学，千万别学ai。 #科技下一站 #还有什么是不能ai的 #与ai同行 #高考 #专业</t>
   </si>
   <si>
     <t>2026-04-29 15:08:15</t>
   </si>
   <si>
-    <t>1-3min视频</t>
-  </si>
-  <si>
-    <t>公开</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>0.025000</t>
-  </si>
-  <si>
-    <t>0.224490</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>0.428571</t>
-  </si>
-  <si>
-    <t>9.632653</t>
+    <t>482</t>
+  </si>
+  <si>
+    <t>0.022774</t>
+  </si>
+  <si>
+    <t>0.366606</t>
+  </si>
+  <si>
+    <t>0.370236</t>
+  </si>
+  <si>
+    <t>15.689655</t>
+  </si>
+  <si>
+    <t>16</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
-    <t>0</t>
+    <t>8</t>
   </si>
   <si>
     <t>家人们，我把AI的价格秘密整理出来了#说真话 #职场干货 #科技下一站 #还有什么是不能ai的 #与ai同行</t>
@@ -108,22 +171,22 @@
     <t>2026-04-29 07:03:00</t>
   </si>
   <si>
-    <t>92</t>
-  </si>
-  <si>
-    <t>0.068182</t>
-  </si>
-  <si>
-    <t>0.312500</t>
-  </si>
-  <si>
-    <t>0.479167</t>
-  </si>
-  <si>
-    <t>13.614583</t>
-  </si>
-  <si>
-    <t>3</t>
+    <t>163</t>
+  </si>
+  <si>
+    <t>0.066265</t>
+  </si>
+  <si>
+    <t>0.324176</t>
+  </si>
+  <si>
+    <t>0.472527</t>
+  </si>
+  <si>
+    <t>14.598901</t>
+  </si>
+  <si>
+    <t>4</t>
   </si>
   <si>
     <t>明明国内算力更稀缺，为什么反而更便 #科技下一站 #与ai同行 #token</t>
@@ -132,34 +195,34 @@
     <t>2026-04-28 19:57:16</t>
   </si>
   <si>
-    <t>5077</t>
-  </si>
-  <si>
-    <t>0.060157</t>
-  </si>
-  <si>
-    <t>0.508917</t>
-  </si>
-  <si>
-    <t>0.283285</t>
-  </si>
-  <si>
-    <t>24.584197</t>
-  </si>
-  <si>
-    <t>77</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>58</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>8</t>
+    <t>8014</t>
+  </si>
+  <si>
+    <t>0.059285</t>
+  </si>
+  <si>
+    <t>0.501034</t>
+  </si>
+  <si>
+    <t>0.290162</t>
+  </si>
+  <si>
+    <t>24.884349</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>119</t>
+  </si>
+  <si>
+    <t>21</t>
   </si>
   <si>
     <t>别人聊 AI 的话题，我连插嘴的资格都没有 #科技下一站 #AI编程 #大模型</t>
@@ -168,22 +231,19 @@
     <t>2026-04-25 22:05:35</t>
   </si>
   <si>
-    <t>198</t>
-  </si>
-  <si>
-    <t>0.010363</t>
-  </si>
-  <si>
-    <t>0.212264</t>
-  </si>
-  <si>
-    <t>0.570755</t>
-  </si>
-  <si>
-    <t>6.375587</t>
-  </si>
-  <si>
-    <t>5</t>
+    <t>202</t>
+  </si>
+  <si>
+    <t>0.010101</t>
+  </si>
+  <si>
+    <t>0.207373</t>
+  </si>
+  <si>
+    <t>0.562212</t>
+  </si>
+  <si>
+    <t>6.293578</t>
   </si>
   <si>
     <t>AI编程不是选修课，是打工人的必修课！ #科技下一站 #AI编程 #大模型 #智能体</t>
@@ -192,27 +252,24 @@
     <t>2026-04-22 11:42:56</t>
   </si>
   <si>
-    <t>117</t>
-  </si>
-  <si>
-    <t>0.024793</t>
-  </si>
-  <si>
-    <t>0.294118</t>
-  </si>
-  <si>
-    <t>0.455882</t>
-  </si>
-  <si>
-    <t>17.227941</t>
+    <t>124</t>
+  </si>
+  <si>
+    <t>0.023256</t>
+  </si>
+  <si>
+    <t>0.300699</t>
+  </si>
+  <si>
+    <t>0.447552</t>
+  </si>
+  <si>
+    <t>16.608392</t>
   </si>
   <si>
     <t>7</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>好险！差点被裁，多亏我学了AI.给0基础的AI入门课，不用担心听不懂、学不会。#这是个真实的事情 #先定一个小目标 #科技下一站 #与ai同行</t>
   </si>
   <si>
@@ -222,19 +279,19 @@
     <t>图文</t>
   </si>
   <si>
-    <t>132</t>
-  </si>
-  <si>
-    <t>0.119048</t>
+    <t>139</t>
+  </si>
+  <si>
+    <t>0.114504</t>
   </si>
   <si>
     <t>0.000000</t>
   </si>
   <si>
-    <t>0.503448</t>
-  </si>
-  <si>
-    <t>4.000000</t>
+    <t>0.506579</t>
+  </si>
+  <si>
+    <t>3.953947</t>
   </si>
   <si>
     <t>郑州龙虾公开课 #抖音科技风向标 #openclaw #郑州 #人工智能</t>
@@ -246,28 +303,25 @@
     <t>1min-视频</t>
   </si>
   <si>
-    <t>1057</t>
-  </si>
-  <si>
-    <t>0.101190</t>
-  </si>
-  <si>
-    <t>0.296207</t>
-  </si>
-  <si>
-    <t>0.394673</t>
-  </si>
-  <si>
-    <t>5.057508</t>
+    <t>1060</t>
+  </si>
+  <si>
+    <t>0.102362</t>
+  </si>
+  <si>
+    <t>0.296563</t>
+  </si>
+  <si>
+    <t>0.395683</t>
+  </si>
+  <si>
+    <t>5.059289</t>
   </si>
   <si>
     <t>13</t>
   </si>
   <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>6</t>
+    <t>51</t>
   </si>
   <si>
     <t>极简三步搭建自己的skills，养龙虾必备 #科技下一站 #超好用的ai指令分享</t>
@@ -279,22 +333,22 @@
     <t>5min+视频</t>
   </si>
   <si>
-    <t>3460</t>
-  </si>
-  <si>
-    <t>0.005468</t>
-  </si>
-  <si>
-    <t>0.183970</t>
-  </si>
-  <si>
-    <t>0.652542</t>
-  </si>
-  <si>
-    <t>0.561323</t>
-  </si>
-  <si>
-    <t>10.164263</t>
+    <t>3556</t>
+  </si>
+  <si>
+    <t>0.005887</t>
+  </si>
+  <si>
+    <t>0.186485</t>
+  </si>
+  <si>
+    <t>0.620968</t>
+  </si>
+  <si>
+    <t>0.558408</t>
+  </si>
+  <si>
+    <t>10.647503</t>
   </si>
   <si>
     <t>25</t>
@@ -309,28 +363,28 @@
     <t>2026-03-31 22:29:00</t>
   </si>
   <si>
-    <t>2289</t>
-  </si>
-  <si>
-    <t>0.012895</t>
-  </si>
-  <si>
-    <t>0.297154</t>
-  </si>
-  <si>
-    <t>0.380282</t>
-  </si>
-  <si>
-    <t>0.431301</t>
-  </si>
-  <si>
-    <t>16.524577</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>11</t>
+    <t>2391</t>
+  </si>
+  <si>
+    <t>0.013434</t>
+  </si>
+  <si>
+    <t>0.300385</t>
+  </si>
+  <si>
+    <t>0.366667</t>
+  </si>
+  <si>
+    <t>0.430385</t>
+  </si>
+  <si>
+    <t>16.635011</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>14</t>
   </si>
   <si>
     <t>23</t>
@@ -342,97 +396,100 @@
     <t>2026-03-26 16:05:44</t>
   </si>
   <si>
-    <t>5650</t>
-  </si>
-  <si>
-    <t>0.031902</t>
-  </si>
-  <si>
-    <t>0.565323</t>
-  </si>
-  <si>
-    <t>0.761421</t>
-  </si>
-  <si>
-    <t>0.252109</t>
-  </si>
-  <si>
-    <t>37.985863</t>
+    <t>5714</t>
+  </si>
+  <si>
+    <t>0.031696</t>
+  </si>
+  <si>
+    <t>0.564984</t>
+  </si>
+  <si>
+    <t>0.763547</t>
+  </si>
+  <si>
+    <t>0.251618</t>
+  </si>
+  <si>
+    <t>38.178702</t>
+  </si>
+  <si>
+    <t>75</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>86</t>
+  </si>
+  <si>
+    <t>284</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>保姆级 WorkBuddy 安装教程！腾讯版龙虾 AI 办公 #openclaw #workbuddy #养龙虾</t>
+  </si>
+  <si>
+    <t>2026-03-26 07:30:00</t>
+  </si>
+  <si>
+    <t>1558</t>
+  </si>
+  <si>
+    <t>0.076014</t>
+  </si>
+  <si>
+    <t>0.494118</t>
+  </si>
+  <si>
+    <t>0.673203</t>
+  </si>
+  <si>
+    <t>0.274020</t>
+  </si>
+  <si>
+    <t>29.113742</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>全流程操作，OpenClaw配置飞书 #openclaw #飞书 #AI #龙虾</t>
+  </si>
+  <si>
+    <t>2026-03-09 07:30:00</t>
+  </si>
+  <si>
+    <t>5727</t>
+  </si>
+  <si>
+    <t>0.010402</t>
+  </si>
+  <si>
+    <t>0.472163</t>
+  </si>
+  <si>
+    <t>0.413919</t>
+  </si>
+  <si>
+    <t>0.267767</t>
+  </si>
+  <si>
+    <t>21.595212</t>
   </si>
   <si>
     <t>74</t>
   </si>
   <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>84</t>
-  </si>
-  <si>
-    <t>281</t>
-  </si>
-  <si>
-    <t>47</t>
-  </si>
-  <si>
-    <t>保姆级 WorkBuddy 安装教程！腾讯版龙虾 AI 办公 #openclaw #workbuddy #养龙虾</t>
-  </si>
-  <si>
-    <t>2026-03-26 07:30:00</t>
-  </si>
-  <si>
-    <t>1495</t>
-  </si>
-  <si>
-    <t>0.074573</t>
-  </si>
-  <si>
-    <t>0.500800</t>
-  </si>
-  <si>
-    <t>0.675497</t>
-  </si>
-  <si>
-    <t>0.278933</t>
-  </si>
-  <si>
-    <t>29.415493</t>
-  </si>
-  <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>全流程操作，OpenClaw配置飞书 #openclaw #飞书 #AI #龙虾</t>
-  </si>
-  <si>
-    <t>2026-03-09 07:30:00</t>
-  </si>
-  <si>
-    <t>5704</t>
-  </si>
-  <si>
-    <t>0.010250</t>
-  </si>
-  <si>
-    <t>0.472915</t>
-  </si>
-  <si>
-    <t>0.411765</t>
-  </si>
-  <si>
-    <t>0.268375</t>
-  </si>
-  <si>
-    <t>21.586615</t>
-  </si>
-  <si>
-    <t>73</t>
-  </si>
-  <si>
     <t>45</t>
   </si>
   <si>
-    <t>160</t>
+    <t>161</t>
   </si>
   <si>
     <t>12</t>
@@ -444,25 +501,22 @@
     <t>2026-03-09 06:35:00</t>
   </si>
   <si>
-    <t>808</t>
-  </si>
-  <si>
-    <t>0.016393</t>
-  </si>
-  <si>
-    <t>0.348865</t>
+    <t>809</t>
+  </si>
+  <si>
+    <t>0.016371</t>
+  </si>
+  <si>
+    <t>0.348449</t>
   </si>
   <si>
     <t>0.653680</t>
   </si>
   <si>
-    <t>0.378734</t>
-  </si>
-  <si>
-    <t>19.284382</t>
-  </si>
-  <si>
-    <t>15</t>
+    <t>0.378282</t>
+  </si>
+  <si>
+    <t>19.264261</t>
   </si>
   <si>
     <t>这就是马六甲海峡吗？这么震撼。#航班 #飞机上 #新加坡</t>
@@ -496,16 +550,16 @@
     <t>2026-02-20 08:05:59</t>
   </si>
   <si>
-    <t>341</t>
-  </si>
-  <si>
-    <t>0.200000</t>
-  </si>
-  <si>
-    <t>0.652174</t>
-  </si>
-  <si>
-    <t>2.689737</t>
+    <t>342</t>
+  </si>
+  <si>
+    <t>0.201550</t>
+  </si>
+  <si>
+    <t>0.651442</t>
+  </si>
+  <si>
+    <t>2.703088</t>
   </si>
   <si>
     <t>在吉隆坡，又住到了人生酒店。#出国旅游 #吉隆坡 #武吉免登</t>
@@ -514,16 +568,16 @@
     <t>2026-02-19 20:37:39</t>
   </si>
   <si>
-    <t>446</t>
-  </si>
-  <si>
-    <t>0.192067</t>
-  </si>
-  <si>
-    <t>0.543726</t>
-  </si>
-  <si>
-    <t>4.334586</t>
+    <t>448</t>
+  </si>
+  <si>
+    <t>0.193347</t>
+  </si>
+  <si>
+    <t>0.543561</t>
+  </si>
+  <si>
+    <t>4.333333</t>
   </si>
   <si>
     <t>9</t>
@@ -553,16 +607,16 @@
     <t>2026-02-19 20:33:31</t>
   </si>
   <si>
-    <t>298</t>
-  </si>
-  <si>
-    <t>0.260450</t>
-  </si>
-  <si>
-    <t>0.432024</t>
-  </si>
-  <si>
-    <t>4.397590</t>
+    <t>299</t>
+  </si>
+  <si>
+    <t>0.262821</t>
+  </si>
+  <si>
+    <t>0.430723</t>
+  </si>
+  <si>
+    <t>4.399399</t>
   </si>
   <si>
     <t>你的AI编程用到什么程度了？用起来吧，朋友们#人工智能 #AI编程 #大模型</t>
@@ -610,19 +664,19 @@
     <t>2026-02-05 19:33:01</t>
   </si>
   <si>
-    <t>238</t>
-  </si>
-  <si>
-    <t>0.037344</t>
-  </si>
-  <si>
-    <t>0.302239</t>
-  </si>
-  <si>
-    <t>0.417910</t>
-  </si>
-  <si>
-    <t>16.527675</t>
+    <t>241</t>
+  </si>
+  <si>
+    <t>0.036735</t>
+  </si>
+  <si>
+    <t>0.305147</t>
+  </si>
+  <si>
+    <t>0.415441</t>
+  </si>
+  <si>
+    <t>16.381818</t>
   </si>
   <si>
     <t>在重庆理工大学分享AI编程工具Trae.#一般人不告诉他 #科技下一站 #AI编程</t>
@@ -670,64 +724,19 @@
     <t>2026-01-31 19:59:43</t>
   </si>
   <si>
-    <t>475</t>
-  </si>
-  <si>
-    <t>0.033932</t>
-  </si>
-  <si>
-    <t>0.163934</t>
-  </si>
-  <si>
-    <t>0.606557</t>
-  </si>
-  <si>
-    <t>5.218412</t>
-  </si>
-  <si>
-    <t>AI是怎么计算的？ #计算 #好书推荐</t>
-  </si>
-  <si>
-    <t>2026-01-30 20:00:00</t>
-  </si>
-  <si>
-    <t>427</t>
-  </si>
-  <si>
-    <t>0.019190</t>
-  </si>
-  <si>
-    <t>0.248092</t>
-  </si>
-  <si>
-    <t>0.522901</t>
-  </si>
-  <si>
-    <t>11.133333</t>
-  </si>
-  <si>
-    <t>越学越流畅，编程就看这个 #python #开发</t>
-  </si>
-  <si>
-    <t>2026-01-29 19:55:00</t>
-  </si>
-  <si>
-    <t>1566</t>
-  </si>
-  <si>
-    <t>0.012353</t>
-  </si>
-  <si>
-    <t>0.251925</t>
-  </si>
-  <si>
-    <t>0.508801</t>
-  </si>
-  <si>
-    <t>6.111661</t>
-  </si>
-  <si>
-    <t>22</t>
+    <t>477</t>
+  </si>
+  <si>
+    <t>0.033797</t>
+  </si>
+  <si>
+    <t>0.161871</t>
+  </si>
+  <si>
+    <t>0.600719</t>
+  </si>
+  <si>
+    <t>5.206835</t>
   </si>
 </sst>
 </file>
@@ -1203,24 +1212,24 @@
         <v>27</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>18</v>
@@ -1229,48 +1238,48 @@
         <v>19</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>27</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>18</v>
@@ -1279,48 +1288,48 @@
         <v>19</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>18</v>
@@ -1329,48 +1338,48 @@
         <v>19</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>18</v>
@@ -1379,87 +1388,87 @@
         <v>19</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>27</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>64</v>
+        <v>38</v>
       </c>
       <c r="L7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M7" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="N7" s="1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>27</v>
@@ -1467,52 +1476,52 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
@@ -1535,772 +1544,772 @@
         <v>88</v>
       </c>
       <c r="G9" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="K9" s="1" t="s">
-        <v>93</v>
+        <v>56</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="H10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="K10" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="L10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="O10" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="N10" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>105</v>
-      </c>
       <c r="P10" s="1" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="K11" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="L11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="O11" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="J11" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>117</v>
-      </c>
       <c r="P11" s="1" t="s">
-        <v>118</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="I12" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="K12" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="L12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="O12" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="L12" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="M12" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N12" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="O12" s="1" t="s">
-        <v>127</v>
-      </c>
       <c r="P12" s="1" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="K13" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="L13" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="M13" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="N13" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="O13" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="P13" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="M13" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="N13" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="O13" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="P13" s="1" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="K14" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="N14" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="O14" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="M14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N14" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="O14" s="1" t="s">
-        <v>139</v>
-      </c>
       <c r="P14" s="1" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="H15" s="1" t="s">
+      <c r="I15" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="K15" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="K15" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="L15" s="1" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>27</v>
+        <v>156</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>81</v>
+        <v>157</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>27</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>70</v>
+        <v>164</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="L16" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>47</v>
+        <v>158</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>70</v>
+        <v>171</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="M17" s="1" t="s">
         <v>27</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>168</v>
+        <v>100</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>81</v>
+        <v>48</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>63</v>
+        <v>186</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="M20" s="1" t="s">
         <v>27</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>23</v>
+        <v>89</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="M21" s="1" t="s">
         <v>27</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>55</v>
+        <v>83</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>23</v>
+        <v>89</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>83</v>
+        <v>38</v>
       </c>
       <c r="L22" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="O22" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M22" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="N22" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="O22" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="P22" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>67</v>
+        <v>94</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>104</v>
+        <v>28</v>
       </c>
       <c r="L23" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="P23" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="N23" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="O23" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="P23" s="1" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="H24" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="M24" s="1" t="s">
         <v>27</v>
@@ -2309,160 +2318,160 @@
         <v>27</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="P24" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>23</v>
+        <v>89</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="N25" s="1" t="s">
         <v>27</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>26</v>
+        <v>112</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>148</v>
+        <v>47</v>
       </c>
       <c r="L26" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>168</v>
+        <v>30</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="H27" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>235</v>
+        <v>29</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="N27" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="O27" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="O27" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="P27" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>